<commit_message>
Update Excel model with interactive fair value calculator sheet
</commit_message>
<xml_diff>
--- a/Zorlu_Enerji_Credit_Model_and_Recovery.xlsx
+++ b/Zorlu_Enerji_Credit_Model_and_Recovery.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generation_Only_Stress" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mgmt_Deficit_Valuation" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zorlu_Group_Contagion" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interactive_Fair_Value_Calc" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="17">
     <numFmt numFmtId="164" formatCode="$#,##0.0"/>
     <numFmt numFmtId="165" formatCode="-0.0%"/>
     <numFmt numFmtId="166" formatCode="($#,##0.0)"/>
@@ -40,8 +41,12 @@
     <numFmt numFmtId="174" formatCode="0.0 'Mo'"/>
     <numFmt numFmtId="175" formatCode="0.00 'x'"/>
     <numFmt numFmtId="176" formatCode="0.0"/>
+    <numFmt numFmtId="177" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="178" formatCode="+$#,##0.00;-$#,##0.00;$0.00"/>
+    <numFmt numFmtId="179" formatCode="0.000x"/>
+    <numFmt numFmtId="180" formatCode="-$#,##0.00"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="36">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -204,8 +209,60 @@
       <color rgb="00C05621"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -284,8 +341,44 @@
         <bgColor rgb="00FFFAF0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF08A"/>
+        <bgColor rgb="00FEF08A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFBF1"/>
+        <bgColor rgb="00CCFBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -414,11 +507,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001E293B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -708,6 +829,68 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="31" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="31" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="30" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="176" fontId="31" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="31" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="33" fillId="16" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="178" fontId="34" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="30" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="34" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="179" fontId="30" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="34" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="180" fontId="30" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="9" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="18" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1371,12 +1554,12 @@
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A8:K8"/>
+    <mergeCell ref="C4:D4"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="I4:K4"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A8:K8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1997,6 +2180,847 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="110" t="inlineStr">
+        <is>
+          <t>Zorlu Enerji Eurobond ($1.1B 11% 2030) — Interactive Restructuring Fair Value Engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="111" t="inlineStr">
+        <is>
+          <t>Yellow cells (B6:B18) are user inputs. Change negotiation time, haircut, extension, or exit yield to calculate implied bond fair value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="112" t="inlineStr">
+        <is>
+          <t>RESTRUCTURING ASSUMPTIONS &amp; INPUTS</t>
+        </is>
+      </c>
+      <c r="F5" s="112" t="inlineStr">
+        <is>
+          <t>SEMI-ANNUAL CASH FLOW SCHEDULE (POST-CLOSING)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="113" t="inlineStr">
+        <is>
+          <t>Negotiation Time to Closing (Months)</t>
+        </is>
+      </c>
+      <c r="C6" s="114" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" s="115" t="inlineStr">
+        <is>
+          <t>Time coupons are frozen; illiquid distressed carry period</t>
+        </is>
+      </c>
+      <c r="F6" s="116" t="inlineStr">
+        <is>
+          <t>Period (t)</t>
+        </is>
+      </c>
+      <c r="G6" s="116" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="H6" s="116" t="inlineStr">
+        <is>
+          <t>Cash Flow ($)</t>
+        </is>
+      </c>
+      <c r="I6" s="116" t="inlineStr">
+        <is>
+          <t>Formula / Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="113" t="inlineStr">
+        <is>
+          <t>Annual Distressed Discount Rate</t>
+        </is>
+      </c>
+      <c r="C7" s="117" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D7" s="115" t="inlineStr">
+        <is>
+          <t>Required holding yield / negative carry penalty during workout</t>
+        </is>
+      </c>
+      <c r="F7" s="118" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="119">
+        <f>F7*0.5</f>
+        <v/>
+      </c>
+      <c r="H7" s="120">
+        <f>IF(F7&gt;(3.5+$C$9)*2, 0, IF(F7&lt;=(3.5+$C$9)*2, IF(F7&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F7-1))*($C$10/2), $C$25*($C$13/2)) + IF(F7=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I7" s="121">
+        <f>IF(F7&gt;(3.5+$C$9)*2, "Matured", IF(F7&lt;=$C$12*2, "PIK Cash Coupon", IF(F7=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="113" t="inlineStr">
+        <is>
+          <t>Nominal Principal Haircut</t>
+        </is>
+      </c>
+      <c r="C8" s="117" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D8" s="115" t="inlineStr">
+        <is>
+          <t>Face value write-down upon exchange offer settlement</t>
+        </is>
+      </c>
+      <c r="F8" s="118" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="119">
+        <f>F8*0.5</f>
+        <v/>
+      </c>
+      <c r="H8" s="120">
+        <f>IF(F8&gt;(3.5+$C$9)*2, 0, IF(F8&lt;=(3.5+$C$9)*2, IF(F8&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F8-1))*($C$10/2), $C$25*($C$13/2)) + IF(F8=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I8" s="121">
+        <f>IF(F8&gt;(3.5+$C$9)*2, "Matured", IF(F8&lt;=$C$12*2, "PIK Cash Coupon", IF(F8=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="113" t="inlineStr">
+        <is>
+          <t>Maturity Extension from 2030 (Years)</t>
+        </is>
+      </c>
+      <c r="C9" s="122" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="115" t="inlineStr">
+        <is>
+          <t>New final maturity tenor = 3.5 yrs remaining + extension</t>
+        </is>
+      </c>
+      <c r="F9" s="118" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="119">
+        <f>F9*0.5</f>
+        <v/>
+      </c>
+      <c r="H9" s="120">
+        <f>IF(F9&gt;(3.5+$C$9)*2, 0, IF(F9&lt;=(3.5+$C$9)*2, IF(F9&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F9-1))*($C$10/2), $C$25*($C$13/2)) + IF(F9=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I9" s="121">
+        <f>IF(F9&gt;(3.5+$C$9)*2, "Matured", IF(F9&lt;=$C$12*2, "PIK Cash Coupon", IF(F9=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="113" t="inlineStr">
+        <is>
+          <t>New Cash Coupon Rate (p.a.)</t>
+        </is>
+      </c>
+      <c r="C10" s="117" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D10" s="115" t="inlineStr">
+        <is>
+          <t>Cash interest paid semi-annually during PIK window</t>
+        </is>
+      </c>
+      <c r="F10" s="118" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="119">
+        <f>F10*0.5</f>
+        <v/>
+      </c>
+      <c r="H10" s="120">
+        <f>IF(F10&gt;(3.5+$C$9)*2, 0, IF(F10&lt;=(3.5+$C$9)*2, IF(F10&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F10-1))*($C$10/2), $C$25*($C$13/2)) + IF(F10=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I10" s="121">
+        <f>IF(F10&gt;(3.5+$C$9)*2, "Matured", IF(F10&lt;=$C$12*2, "PIK Cash Coupon", IF(F10=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="113" t="inlineStr">
+        <is>
+          <t>PIK Coupon Rate (p.a.)</t>
+        </is>
+      </c>
+      <c r="C11" s="117" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="D11" s="115" t="inlineStr">
+        <is>
+          <t>Interest compounded semi-annually into principal face</t>
+        </is>
+      </c>
+      <c r="F11" s="118" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="119">
+        <f>F11*0.5</f>
+        <v/>
+      </c>
+      <c r="H11" s="120">
+        <f>IF(F11&gt;(3.5+$C$9)*2, 0, IF(F11&lt;=(3.5+$C$9)*2, IF(F11&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F11-1))*($C$10/2), $C$25*($C$13/2)) + IF(F11=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I11" s="121">
+        <f>IF(F11&gt;(3.5+$C$9)*2, "Matured", IF(F11&lt;=$C$12*2, "PIK Cash Coupon", IF(F11=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="113" t="inlineStr">
+        <is>
+          <t>PIK Window Duration (Years)</t>
+        </is>
+      </c>
+      <c r="C12" s="122" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="115" t="inlineStr">
+        <is>
+          <t>Years during which PIK coupon compounds</t>
+        </is>
+      </c>
+      <c r="F12" s="118" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="119">
+        <f>F12*0.5</f>
+        <v/>
+      </c>
+      <c r="H12" s="120">
+        <f>IF(F12&gt;(3.5+$C$9)*2, 0, IF(F12&lt;=(3.5+$C$9)*2, IF(F12&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F12-1))*($C$10/2), $C$25*($C$13/2)) + IF(F12=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I12" s="121">
+        <f>IF(F12&gt;(3.5+$C$9)*2, "Matured", IF(F12&lt;=$C$12*2, "PIK Cash Coupon", IF(F12=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="113" t="inlineStr">
+        <is>
+          <t>Post-PIK Step-up Cash Coupon (p.a.)</t>
+        </is>
+      </c>
+      <c r="C13" s="117" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="D13" s="115" t="inlineStr">
+        <is>
+          <t>Cash coupon after PIK window terminates until maturity</t>
+        </is>
+      </c>
+      <c r="F13" s="118" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" s="119">
+        <f>F13*0.5</f>
+        <v/>
+      </c>
+      <c r="H13" s="120">
+        <f>IF(F13&gt;(3.5+$C$9)*2, 0, IF(F13&lt;=(3.5+$C$9)*2, IF(F13&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F13-1))*($C$10/2), $C$25*($C$13/2)) + IF(F13=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I13" s="121">
+        <f>IF(F13&gt;(3.5+$C$9)*2, "Matured", IF(F13&lt;=$C$12*2, "PIK Cash Coupon", IF(F13=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="113" t="inlineStr">
+        <is>
+          <t>Advisory &amp; Legal Fee Friction</t>
+        </is>
+      </c>
+      <c r="C14" s="117" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="D14" s="115" t="inlineStr">
+        <is>
+          <t>Houlihan Lokey, Servo, creditor counsel (leakage from debt)</t>
+        </is>
+      </c>
+      <c r="F14" s="118" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="119">
+        <f>F14*0.5</f>
+        <v/>
+      </c>
+      <c r="H14" s="120">
+        <f>IF(F14&gt;(3.5+$C$9)*2, 0, IF(F14&lt;=(3.5+$C$9)*2, IF(F14&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F14-1))*($C$10/2), $C$25*($C$13/2)) + IF(F14=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I14" s="121">
+        <f>IF(F14&gt;(3.5+$C$9)*2, "Matured", IF(F14&lt;=$C$12*2, "PIK Cash Coupon", IF(F14=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="113" t="inlineStr">
+        <is>
+          <t>Upfront Consent Sweetener Fee</t>
+        </is>
+      </c>
+      <c r="C15" s="117" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D15" s="115" t="inlineStr">
+        <is>
+          <t>Early bird cash fee paid to consenting bondholders at closing</t>
+        </is>
+      </c>
+      <c r="F15" s="118" t="n">
+        <v>9</v>
+      </c>
+      <c r="G15" s="119">
+        <f>F15*0.5</f>
+        <v/>
+      </c>
+      <c r="H15" s="120">
+        <f>IF(F15&gt;(3.5+$C$9)*2, 0, IF(F15&lt;=(3.5+$C$9)*2, IF(F15&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F15-1))*($C$10/2), $C$25*($C$13/2)) + IF(F15=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I15" s="121">
+        <f>IF(F15&gt;(3.5+$C$9)*2, "Matured", IF(F15&lt;=$C$12*2, "PIK Cash Coupon", IF(F15=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="113" t="inlineStr">
+        <is>
+          <t>Asset Sweep Cash Paydown ($ per 100 face)</t>
+        </is>
+      </c>
+      <c r="C16" s="123" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="115" t="inlineStr">
+        <is>
+          <t>Immediate pro-rata debt paydown from non-core sales (ZES/Pak)</t>
+        </is>
+      </c>
+      <c r="F16" s="118" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="119">
+        <f>F16*0.5</f>
+        <v/>
+      </c>
+      <c r="H16" s="120">
+        <f>IF(F16&gt;(3.5+$C$9)*2, 0, IF(F16&lt;=(3.5+$C$9)*2, IF(F16&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F16-1))*($C$10/2), $C$25*($C$13/2)) + IF(F16=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I16" s="121">
+        <f>IF(F16&gt;(3.5+$C$9)*2, "Matured", IF(F16&lt;=$C$12*2, "PIK Cash Coupon", IF(F16=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="113" t="inlineStr">
+        <is>
+          <t>Post-Restructuring Exit Yield (YTM)</t>
+        </is>
+      </c>
+      <c r="C17" s="117" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="D17" s="115" t="inlineStr">
+        <is>
+          <t>Market discount yield for new stabilized bond at emergence</t>
+        </is>
+      </c>
+      <c r="F17" s="118" t="n">
+        <v>11</v>
+      </c>
+      <c r="G17" s="119">
+        <f>F17*0.5</f>
+        <v/>
+      </c>
+      <c r="H17" s="120">
+        <f>IF(F17&gt;(3.5+$C$9)*2, 0, IF(F17&lt;=(3.5+$C$9)*2, IF(F17&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F17-1))*($C$10/2), $C$25*($C$13/2)) + IF(F17=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I17" s="121">
+        <f>IF(F17&gt;(3.5+$C$9)*2, "Matured", IF(F17&lt;=$C$12*2, "PIK Cash Coupon", IF(F17=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="113" t="inlineStr">
+        <is>
+          <t>Current Secondary Market Price</t>
+        </is>
+      </c>
+      <c r="C18" s="123" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="D18" s="115" t="inlineStr">
+        <is>
+          <t>Current secondary broker quote (cents on the dollar)</t>
+        </is>
+      </c>
+      <c r="F18" s="118" t="n">
+        <v>12</v>
+      </c>
+      <c r="G18" s="119">
+        <f>F18*0.5</f>
+        <v/>
+      </c>
+      <c r="H18" s="120">
+        <f>IF(F18&gt;(3.5+$C$9)*2, 0, IF(F18&lt;=(3.5+$C$9)*2, IF(F18&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F18-1))*($C$10/2), $C$25*($C$13/2)) + IF(F18=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I18" s="121">
+        <f>IF(F18&gt;(3.5+$C$9)*2, "Matured", IF(F18&lt;=$C$12*2, "PIK Cash Coupon", IF(F18=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="F19" s="118" t="n">
+        <v>13</v>
+      </c>
+      <c r="G19" s="119">
+        <f>F19*0.5</f>
+        <v/>
+      </c>
+      <c r="H19" s="120">
+        <f>IF(F19&gt;(3.5+$C$9)*2, 0, IF(F19&lt;=(3.5+$C$9)*2, IF(F19&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F19-1))*($C$10/2), $C$25*($C$13/2)) + IF(F19=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I19" s="121">
+        <f>IF(F19&gt;(3.5+$C$9)*2, "Matured", IF(F19&lt;=$C$12*2, "PIK Cash Coupon", IF(F19=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="112" t="inlineStr">
+        <is>
+          <t>MODEL VALUATION &amp; TRADE SIGNALS</t>
+        </is>
+      </c>
+      <c r="F20" s="118" t="n">
+        <v>14</v>
+      </c>
+      <c r="G20" s="119">
+        <f>F20*0.5</f>
+        <v/>
+      </c>
+      <c r="H20" s="120">
+        <f>IF(F20&gt;(3.5+$C$9)*2, 0, IF(F20&lt;=(3.5+$C$9)*2, IF(F20&lt;=$C$12*2, ($C$24*(1+$C$11/2)^(F20-1))*($C$10/2), $C$25*($C$13/2)) + IF(F20=ROUND((3.5+$C$9)*2,0), $C$25, 0), 0))</f>
+        <v/>
+      </c>
+      <c r="I20" s="121">
+        <f>IF(F20&gt;(3.5+$C$9)*2, "Matured", IF(F20&lt;=$C$12*2, "PIK Cash Coupon", IF(F20=ROUND((3.5+$C$9)*2,0), "Coupon + Principal Bullet", "Post-PIK Cash Coupon")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="124" t="inlineStr">
+        <is>
+          <t>IMPLIED FAIR VALUE TODAY (¢ on dollar)</t>
+        </is>
+      </c>
+      <c r="C21" s="125">
+        <f>C29/C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="126" t="inlineStr">
+        <is>
+          <t>Secondary Market Spread (Delta)</t>
+        </is>
+      </c>
+      <c r="C22" s="127">
+        <f>C21-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="126" t="inlineStr">
+        <is>
+          <t>Trade Recommendation Signal</t>
+        </is>
+      </c>
+      <c r="C23" s="128">
+        <f>IF(C22&lt;-3.0, "OVERVALUED / WAIT", IF(C22&gt;3.0, "UNDERVALUED / BUY", "FAIRLY PRICED"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="113" t="inlineStr">
+        <is>
+          <t>New Initial Face Value ($)</t>
+        </is>
+      </c>
+      <c r="C24" s="129">
+        <f>100*(1-C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="113" t="inlineStr">
+        <is>
+          <t>Compounded Face Value post-PIK ($)</t>
+        </is>
+      </c>
+      <c r="C25" s="129">
+        <f>C24*(1+C11/2)^(C12*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="126" t="inlineStr">
+        <is>
+          <t>Present Value of Restructured Bond at Exit ($)</t>
+        </is>
+      </c>
+      <c r="C26" s="130">
+        <f>NPV(C17/2, G7:G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="113" t="inlineStr">
+        <is>
+          <t>Upfront Cash Received (Consent + Sweep) ($)</t>
+        </is>
+      </c>
+      <c r="C27" s="129">
+        <f>100*C15+C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="113" t="inlineStr">
+        <is>
+          <t>Less: Advisory &amp; Friction Drag ($)</t>
+        </is>
+      </c>
+      <c r="C28" s="129">
+        <f>100*C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="126" t="inlineStr">
+        <is>
+          <t>Total Realized Recovery at Closing ($)</t>
+        </is>
+      </c>
+      <c r="C29" s="130">
+        <f>C26+C27-C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="113" t="inlineStr">
+        <is>
+          <t>Negotiation Time Decay Factor</t>
+        </is>
+      </c>
+      <c r="C30" s="131">
+        <f>(1+C7)^(C6/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="126" t="inlineStr">
+        <is>
+          <t>Holding Period IRR to Closing (p.a.)</t>
+        </is>
+      </c>
+      <c r="C31" s="132">
+        <f>(C29/C18)^(12/C6)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="113" t="inlineStr">
+        <is>
+          <t>Carry Drag / Frozen Coupon Penalty ($)</t>
+        </is>
+      </c>
+      <c r="C32" s="133">
+        <f>C21-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="112" t="inlineStr">
+        <is>
+          <t>SENSITIVITY MATRIX: FAIR VALUE TODAY (¢) VS. HAIRCUT AND NEGOTIATION TIME</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="134" t="inlineStr">
+        <is>
+          <t>Months \ Haircut</t>
+        </is>
+      </c>
+      <c r="C36" s="135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="135" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E36" s="135" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F36" s="135" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G36" s="135" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H36" s="135" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="136" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C37" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+      <c r="D37" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+      <c r="E37" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+      <c r="F37" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+      <c r="G37" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+      <c r="H37" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(3/12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="136" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="C38" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+      <c r="D38" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+      <c r="E38" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+      <c r="F38" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+      <c r="G38" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+      <c r="H38" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(6/12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="136" t="inlineStr">
+        <is>
+          <t>8 Months</t>
+        </is>
+      </c>
+      <c r="C39" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+      <c r="D39" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+      <c r="E39" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+      <c r="F39" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+      <c r="G39" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+      <c r="H39" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(8/12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="136" t="inlineStr">
+        <is>
+          <t>12 Months</t>
+        </is>
+      </c>
+      <c r="C40" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+      <c r="D40" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+      <c r="E40" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+      <c r="F40" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+      <c r="G40" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+      <c r="H40" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(12/12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="136" t="inlineStr">
+        <is>
+          <t>18 Months</t>
+        </is>
+      </c>
+      <c r="C41" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+      <c r="D41" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+      <c r="E41" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+      <c r="F41" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+      <c r="G41" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+      <c r="H41" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(18/12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="136" t="inlineStr">
+        <is>
+          <t>24 Months</t>
+        </is>
+      </c>
+      <c r="C42" s="137">
+        <f>($C$29*(1 - (C$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+      <c r="D42" s="137">
+        <f>($C$29*(1 - (D$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+      <c r="E42" s="137">
+        <f>($C$29*(1 - (E$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+      <c r="F42" s="137">
+        <f>($C$29*(1 - (F$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+      <c r="G42" s="137">
+        <f>($C$29*(1 - (G$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+      <c r="H42" s="137">
+        <f>($C$29*(1 - (H$36 - $C$8)*0.85)) / ((1 + $C$7)^(24/12))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7734,59 +8758,39 @@
 4. TIMELINE EXTENDS TO 14 - 18 MONTHS: Unlike a simple coupon reprofiling (which takes 6-9 months), carving out generation assets requires unbundling shared guarantees and securing EPDK regulatory approvals for transferring generation licenses across 10+ plants.</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
+      <c r="B29" s="66" t="n"/>
+      <c r="C29" s="66" t="n"/>
+      <c r="D29" s="66" t="n"/>
+      <c r="E29" s="66" t="n"/>
+      <c r="F29" s="67" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="n"/>
+      <c r="A30" s="68" t="n"/>
+      <c r="F30" s="69" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
+      <c r="A31" s="68" t="n"/>
+      <c r="F31" s="69" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
+      <c r="A32" s="68" t="n"/>
+      <c r="F32" s="69" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
+      <c r="A33" s="68" t="n"/>
+      <c r="F33" s="69" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
+      <c r="A34" s="68" t="n"/>
+      <c r="F34" s="69" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-      <c r="D35" s="4" t="n"/>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="n"/>
+      <c r="A35" s="70" t="n"/>
+      <c r="B35" s="71" t="n"/>
+      <c r="C35" s="71" t="n"/>
+      <c r="D35" s="71" t="n"/>
+      <c r="E35" s="71" t="n"/>
+      <c r="F35" s="72" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>